<commit_message>
Add separate phone banners, softer banner gradient on phones, update image plan sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/iDermaCare-image-content-plan.xlsx
+++ b/docs/iDermaCare-image-content-plan.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Content plan'!$A$1:$U$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Content plan'!$A$1:$U$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -788,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1232,12 +1232,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Hero banner slides</t>
+          <t>Hero banner slides - desktop and tablet</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Large rotating banner at the top of the home page (3 slides).</t>
+          <t>Large rotating banner at the top of the home page (3 slides) for computers and tablets (750 px wide and up).</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Shown 624 px tall on desktop, 546 on tablet, 416 on phone and always cropped to fill, so a phone sees only the centre. Put the product and any text in the middle ~50% of the width; leave the left third calmer because the headline sits there. No text baked into the image - the site adds the headline and button.</t>
+          <t>Shown 624 px tall on desktop and 546 on tablet, always cropped to fill. Put the product in the middle and right; leave the left third calmer because the headline sits there. No text baked into the image - the site adds the headline and button. Phones use the separate phone version below.</t>
         </is>
       </c>
       <c r="N6" s="10" t="inlineStr">
@@ -1298,7 +1298,7 @@
       <c r="T6" s="12" t="n"/>
       <c r="U6" s="10" t="inlineStr"/>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7" ht="84" customHeight="1">
       <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
@@ -1309,28 +1309,28 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Category circles (stories row)</t>
+          <t>Hero banner slides - phone version</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Round pictures under the header: SADOER, Hero, SOME BY MI, Masks, Toners, Patches.</t>
+          <t>Separate tall banner shown on phones (screens under 750 px wide). Optional: if empty, the desktop banner is cropped instead. Set in Admin &gt; Website content &gt; Banner picture for phones.</t>
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>800</v>
+        <v>1080</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>800</v>
+        <v>1440</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>400</v>
+        <v>720</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>400</v>
+        <v>960</v>
       </c>
       <c r="J7" s="8">
         <f>IF(OR(G7="",G7=0),"",ROUND(F7/G7,2)&amp;" : 1")</f>
@@ -1338,30 +1338,26 @@
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>JPG or PNG</t>
+          <t>JPG (or WebP)</t>
         </is>
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>150 KB each</t>
+          <t>300 KB each</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>Square. The site crops it into a circle, so keep the subject centred with space around it. Clean, bright background.</t>
+          <t>Portrait 3:4. Shown about 390 px wide and at least 520 px tall. Put the product in the upper 60%; the bottom 35% sits under the headline and button (a soft dark fade is added by the site), so keep it calm there. No text baked into the image.</t>
         </is>
       </c>
       <c r="N7" s="10" t="inlineStr">
         <is>
-          <t>products/*/1 and 2 (product photos reused)</t>
-        </is>
-      </c>
-      <c r="O7" s="11" t="n">
-        <v>1500</v>
-      </c>
-      <c r="P7" s="11" t="n">
-        <v>1500</v>
-      </c>
+          <t>(none yet)</t>
+        </is>
+      </c>
+      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
       <c r="Q7" s="8">
         <f>IF(O7="","Missing",IF(AND(O7&gt;=H7,P7&gt;=I7),"OK","Too small"))</f>
         <v/>
@@ -1386,28 +1382,28 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Story full-screen photos</t>
+          <t>Category circles (stories row)</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Photo/video that opens when a category circle is tapped (phone-style full screen).</t>
+          <t>Round pictures under the header: SADOER, Hero, SOME BY MI, Masks, Toners, Patches.</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
         <v>6</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>1080</v>
+        <v>800</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>1920</v>
+        <v>800</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>720</v>
+        <v>400</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>1280</v>
+        <v>400</v>
       </c>
       <c r="J8" s="8">
         <f>IF(OR(G8="",G8=0),"",ROUND(F8/G8,2)&amp;" : 1")</f>
@@ -1415,29 +1411,29 @@
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>JPG, or MP4 for video</t>
+          <t>JPG or PNG</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>500 KB photo / 40 MB video</t>
+          <t>150 KB each</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>Portrait 9:16. Keep faces and products away from the top 12% and bottom 18% (buttons and title overlap there).</t>
+          <t>Square. The site crops it into a circle, so keep the subject centred with space around it. Clean, bright background.</t>
         </is>
       </c>
       <c r="N8" s="10" t="inlineStr">
         <is>
-          <t>products/*/1 (product photos reused)</t>
+          <t>products/*/1 and 2 (product photos reused)</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>522</v>
+        <v>1500</v>
       </c>
       <c r="P8" s="11" t="n">
-        <v>624</v>
+        <v>1500</v>
       </c>
       <c r="Q8" s="8">
         <f>IF(O8="","Missing",IF(AND(O8&gt;=H8,P8&gt;=I8),"OK","Too small"))</f>
@@ -1463,28 +1459,28 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Brand logos row</t>
+          <t>Story full-screen photos</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Logos of SADOER, Hero Cosmetics and SOME BY MI in a row, shown as circles.</t>
+          <t>Photo/video that opens when a category circle is tapped (phone-style full screen).</t>
         </is>
       </c>
       <c r="E9" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>800</v>
+        <v>1080</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>800</v>
+        <v>1920</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>400</v>
+        <v>720</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>400</v>
+        <v>1280</v>
       </c>
       <c r="J9" s="8">
         <f>IF(OR(G9="",G9=0),"",ROUND(F9/G9,2)&amp;" : 1")</f>
@@ -1492,26 +1488,30 @@
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>SVG or PNG (transparent)</t>
+          <t>JPG, or MP4 for video</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>100 KB each</t>
+          <t>500 KB photo / 40 MB video</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>Square canvas, logo centred with 15% padding. Use the official brand artwork where you are allowed to.</t>
+          <t>Portrait 9:16. Keep faces and products away from the top 12% and bottom 18% (buttons and title overlap there).</t>
         </is>
       </c>
       <c r="N9" s="10" t="inlineStr">
         <is>
-          <t>brands/sadoer.svg, hero.svg, some-by-mi.svg</t>
-        </is>
-      </c>
-      <c r="O9" s="11" t="n"/>
-      <c r="P9" s="11" t="n"/>
+          <t>products/*/1 (product photos reused)</t>
+        </is>
+      </c>
+      <c r="O9" s="11" t="n">
+        <v>522</v>
+      </c>
+      <c r="P9" s="11" t="n">
+        <v>624</v>
+      </c>
       <c r="Q9" s="8">
         <f>IF(O9="","Missing",IF(AND(O9&gt;=H9,P9&gt;=I9),"OK","Too small"))</f>
         <v/>
@@ -1536,28 +1536,28 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>"Our story" photo</t>
+          <t>Brand logos row</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Picture beside the "A short list, chosen carefully" text.</t>
+          <t>Logos of SADOER, Hero Cosmetics and SOME BY MI in a row, shown as circles.</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="J10" s="8">
         <f>IF(OR(G10="",G10=0),"",ROUND(F10/G10,2)&amp;" : 1")</f>
@@ -1565,30 +1565,26 @@
       </c>
       <c r="K10" s="9" t="inlineStr">
         <is>
-          <t>JPG</t>
+          <t>SVG or PNG (transparent)</t>
         </is>
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>300 KB</t>
+          <t>100 KB each</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Square 1:1. Best as a group shot of the three products on a clean surface.</t>
+          <t>Square canvas, logo centred with 15% padding. Use the official brand artwork where you are allowed to.</t>
         </is>
       </c>
       <c r="N10" s="10" t="inlineStr">
         <is>
-          <t>products/story-trio.jpg</t>
-        </is>
-      </c>
-      <c r="O10" s="11" t="n">
-        <v>1024</v>
-      </c>
-      <c r="P10" s="11" t="n">
-        <v>1024</v>
-      </c>
+          <t>brands/sadoer.svg, hero.svg, some-by-mi.svg</t>
+        </is>
+      </c>
+      <c r="O10" s="11" t="n"/>
+      <c r="P10" s="11" t="n"/>
       <c r="Q10" s="8">
         <f>IF(O10="","Missing",IF(AND(O10&gt;=H10,P10&gt;=I10),"OK","Too small"))</f>
         <v/>
@@ -1613,28 +1609,28 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Customer review photos</t>
+          <t>"Our story" photo</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Photos in the scrolling reviews strip.</t>
+          <t>Picture beside the "A short list, chosen carefully" text.</t>
         </is>
       </c>
       <c r="E11" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F11" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H11" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="I11" s="8" t="n">
         <v>800</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>400</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>400</v>
       </c>
       <c r="J11" s="8">
         <f>IF(OR(G11="",G11=0),"",ROUND(F11/G11,2)&amp;" : 1")</f>
@@ -1647,17 +1643,17 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>200 KB each</t>
+          <t>300 KB</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>Square 1:1 customer photos or product-in-use shots. Only use photos you have permission to show.</t>
+          <t>Square 1:1. Best as a group shot of the three products on a clean surface.</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">
         <is>
-          <t>reviews/review-1 to 8.jpg</t>
+          <t>products/story-trio.jpg</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
@@ -1685,33 +1681,33 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Home / Shop</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Product cards</t>
+          <t>Customer review photos</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Square product picture on every product card (uses the first gallery photo of each product).</t>
+          <t>Photos in the scrolling reviews strip.</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="J12" s="8">
         <f>IF(OR(G12="",G12=0),"",ROUND(F12/G12,2)&amp;" : 1")</f>
@@ -1719,29 +1715,29 @@
       </c>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>JPG or PNG</t>
+          <t>JPG</t>
         </is>
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>300 KB each</t>
+          <t>200 KB each</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Square 1:1, product centred on a plain white or soft background. The first gallery photo is used here, so make it the best one.</t>
+          <t>Square 1:1 customer photos or product-in-use shots. Only use photos you have permission to show.</t>
         </is>
       </c>
       <c r="N12" s="10" t="inlineStr">
         <is>
-          <t>products/*/1 (first gallery photo)</t>
+          <t>reviews/review-1 to 8.jpg</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>800</v>
+        <v>1024</v>
       </c>
       <c r="P12" s="11" t="n">
-        <v>800</v>
+        <v>1024</v>
       </c>
       <c r="Q12" s="8">
         <f>IF(O12="","Missing",IF(AND(O12&gt;=H12,P12&gt;=I12),"OK","Too small"))</f>
@@ -1762,33 +1758,33 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Product pages</t>
+          <t>Home / Shop</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Main product photo (gallery photo 1)</t>
+          <t>Product cards</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Big picture at the top of each product page; zoomable.</t>
+          <t>Square product picture on every product card (uses the first gallery photo of each product).</t>
         </is>
       </c>
       <c r="E13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="J13" s="8">
         <f>IF(OR(G13="",G13=0),"",ROUND(F13/G13,2)&amp;" : 1")</f>
@@ -1796,29 +1792,29 @@
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>JPG (PNG if transparent)</t>
+          <t>JPG or PNG</t>
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>500 KB each</t>
+          <t>300 KB each</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Square 1:1, product fills about 80% of the frame on a white background. Sharp label text. Shown with 24 px padding, so do not crop tight.</t>
+          <t>Square 1:1, product centred on a plain white or soft background. The first gallery photo is used here, so make it the best one.</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
         <is>
-          <t>products/*/1</t>
+          <t>products/*/1 (first gallery photo)</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>522</v>
+        <v>800</v>
       </c>
       <c r="P13" s="11" t="n">
-        <v>624</v>
+        <v>800</v>
       </c>
       <c r="Q13" s="8">
         <f>IF(O13="","Missing",IF(AND(O13&gt;=H13,P13&gt;=I13),"OK","Too small"))</f>
@@ -1833,7 +1829,7 @@
       <c r="T13" s="12" t="n"/>
       <c r="U13" s="10" t="inlineStr"/>
     </row>
-    <row r="14" ht="56" customHeight="1">
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="8" t="n">
         <v>13</v>
       </c>
@@ -1844,16 +1840,16 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Extra gallery photos</t>
+          <t>Main product photo (gallery photo 1)</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Pictures 2 to 6 for each product: pack front/back, texture, size comparison, how to use, ingredients / label.</t>
+          <t>Big picture at the top of each product page; zoomable.</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>2000</v>
@@ -1873,7 +1869,7 @@
       </c>
       <c r="K14" s="9" t="inlineStr">
         <is>
-          <t>JPG</t>
+          <t>JPG (PNG if transparent)</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">
@@ -1883,19 +1879,19 @@
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>5 extra photos per product (3 products). Square 1:1. Mix: close-up of the texture, product in hand for scale, step-by-step use, the back label, one lifestyle photo.</t>
+          <t>Square 1:1, product fills about 80% of the frame on a white background. Sharp label text. Shown with 24 px padding, so do not crop tight.</t>
         </is>
       </c>
       <c r="N14" s="10" t="inlineStr">
         <is>
-          <t>products/*/2 to 7</t>
+          <t>products/*/1</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
         <v>522</v>
       </c>
       <c r="P14" s="11" t="n">
-        <v>522</v>
+        <v>624</v>
       </c>
       <c r="Q14" s="8">
         <f>IF(O14="","Missing",IF(AND(O14&gt;=H14,P14&gt;=I14),"OK","Too small"))</f>
@@ -1910,7 +1906,7 @@
       <c r="T14" s="12" t="n"/>
       <c r="U14" s="10" t="inlineStr"/>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="56" customHeight="1">
       <c r="A15" s="8" t="n">
         <v>14</v>
       </c>
@@ -1921,28 +1917,28 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Product video (landscape)</t>
+          <t>Extra gallery photos</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Short demo or brand video in the player on the product page.</t>
+          <t>Pictures 2 to 6 for each product: pack front/back, texture, size comparison, how to use, ingredients / label.</t>
         </is>
       </c>
       <c r="E15" s="8" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>1920</v>
+        <v>2000</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>1080</v>
+        <v>2000</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>1280</v>
+        <v>1000</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>720</v>
+        <v>1000</v>
       </c>
       <c r="J15" s="8">
         <f>IF(OR(G15="",G15=0),"",ROUND(F15/G15,2)&amp;" : 1")</f>
@@ -1950,26 +1946,30 @@
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>MP4 (H.264)</t>
+          <t>JPG</t>
         </is>
       </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
-          <t>40 MB</t>
+          <t>500 KB each</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>16:9, 15-45 seconds, with a poster frame. Add captions: many people watch without sound.</t>
+          <t>5 extra photos per product (3 products). Square 1:1. Mix: close-up of the texture, product in hand for scale, step-by-step use, the back label, one lifestyle photo.</t>
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr">
         <is>
-          <t>videos/sadoer.mp4, mighty-patch.mp4, some-by-mi.mp4</t>
-        </is>
-      </c>
-      <c r="O15" s="11" t="n"/>
-      <c r="P15" s="11" t="n"/>
+          <t>products/*/2 to 7</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="n">
+        <v>522</v>
+      </c>
+      <c r="P15" s="11" t="n">
+        <v>522</v>
+      </c>
       <c r="Q15" s="8">
         <f>IF(O15="","Missing",IF(AND(O15&gt;=H15,P15&gt;=I15),"OK","Too small"))</f>
         <v/>
@@ -1994,28 +1994,28 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Short vertical videos</t>
+          <t>Product video (landscape)</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Optional short video for the story / reels style viewer.</t>
+          <t>Short demo or brand video in the player on the product page.</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
         <v>3</v>
       </c>
       <c r="F16" s="8" t="n">
+        <v>1920</v>
+      </c>
+      <c r="G16" s="8" t="n">
         <v>1080</v>
       </c>
-      <c r="G16" s="8" t="n">
-        <v>1920</v>
-      </c>
       <c r="H16" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="I16" s="8" t="n">
         <v>720</v>
-      </c>
-      <c r="I16" s="8" t="n">
-        <v>1280</v>
       </c>
       <c r="J16" s="8">
         <f>IF(OR(G16="",G16=0),"",ROUND(F16/G16,2)&amp;" : 1")</f>
@@ -2033,12 +2033,12 @@
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>9:16, 10-30 seconds. Key action in the middle of the frame.</t>
+          <t>16:9, 15-45 seconds, with a poster frame. Add captions: many people watch without sound.</t>
         </is>
       </c>
       <c r="N16" s="10" t="inlineStr">
         <is>
-          <t>(none)</t>
+          <t>videos/sadoer.mp4, mighty-patch.mp4, some-by-mi.mp4</t>
         </is>
       </c>
       <c r="O16" s="11" t="n"/>
@@ -2062,33 +2062,33 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Cart / Checkout</t>
+          <t>Product pages</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Cart thumbnails</t>
+          <t>Short vertical videos</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Small product picture in the cart (88 x 88 px).</t>
+          <t>Optional short video for the story / reels style viewer.</t>
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>400</v>
+        <v>1080</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>400</v>
+        <v>1920</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>200</v>
+        <v>720</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>200</v>
+        <v>1280</v>
       </c>
       <c r="J17" s="8">
         <f>IF(OR(G17="",G17=0),"",ROUND(F17/G17,2)&amp;" : 1")</f>
@@ -2096,34 +2096,33 @@
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>Automatic</t>
+          <t>MP4 (H.264)</t>
         </is>
       </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>40 MB</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>No extra picture needed: the first product gallery photo is reused.</t>
+          <t>9:16, 10-30 seconds. Key action in the middle of the frame.</t>
         </is>
       </c>
       <c r="N17" s="10" t="inlineStr">
         <is>
-          <t>(automatic)</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="O17" s="11" t="n"/>
       <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="8" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+      <c r="Q17" s="8">
+        <f>IF(O17="","Missing",IF(AND(O17&gt;=H17,P17&gt;=I17),"OK","Too small"))</f>
+        <v/>
       </c>
       <c r="R17" s="11" t="inlineStr">
         <is>
-          <t>Not needed</t>
+          <t>To do</t>
         </is>
       </c>
       <c r="S17" s="10" t="inlineStr"/>
@@ -2136,33 +2135,33 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>About</t>
+          <t>Cart / Checkout</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>About us photo</t>
+          <t>Cart thumbnails</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Photo on the About page: the team, the office or the story.</t>
+          <t>Small product picture in the cart (88 x 88 px).</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>1067</v>
+        <v>400</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>1200</v>
+        <v>200</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="J18" s="8">
         <f>IF(OR(G18="",G18=0),"",ROUND(F18/G18,2)&amp;" : 1")</f>
@@ -2170,37 +2169,34 @@
       </c>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>JPG</t>
+          <t>Automatic</t>
         </is>
       </c>
       <c r="L18" s="9" t="inlineStr">
         <is>
-          <t>400 KB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Landscape 3:2 works best. It is shown whole (not cropped), so any shape will fit, but wide photos fill the page better.</t>
+          <t>No extra picture needed: the first product gallery photo is reused.</t>
         </is>
       </c>
       <c r="N18" s="10" t="inlineStr">
         <is>
-          <t>about/iderma-care.png</t>
-        </is>
-      </c>
-      <c r="O18" s="11" t="n">
-        <v>1024</v>
-      </c>
-      <c r="P18" s="11" t="n">
-        <v>1024</v>
-      </c>
-      <c r="Q18" s="8">
-        <f>IF(O18="","Missing",IF(AND(O18&gt;=H18,P18&gt;=I18),"OK","Too small"))</f>
-        <v/>
+          <t>(automatic)</t>
+        </is>
+      </c>
+      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="11" t="n"/>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
       <c r="R18" s="11" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Not needed</t>
         </is>
       </c>
       <c r="S18" s="10" t="inlineStr"/>
@@ -2213,33 +2209,33 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>About</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Blog cover images</t>
+          <t>About us photo</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>A cover picture for each article (the site does not show one yet; a small code change adds it).</t>
+          <t>Photo on the About page: the team, the office or the story.</t>
         </is>
       </c>
       <c r="E19" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>630</v>
+        <v>1067</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>1200</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>630</v>
+        <v>800</v>
       </c>
       <c r="J19" s="8">
         <f>IF(OR(G19="",G19=0),"",ROUND(F19/G19,2)&amp;" : 1")</f>
@@ -2252,21 +2248,25 @@
       </c>
       <c r="L19" s="9" t="inlineStr">
         <is>
-          <t>250 KB each</t>
+          <t>400 KB</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Landscape 1.91:1, one per post, no text baked in. Also used as the link preview image when the article is shared.</t>
+          <t>Landscape 3:2 works best. It is shown whole (not cropped), so any shape will fit, but wide photos fill the page better.</t>
         </is>
       </c>
       <c r="N19" s="10" t="inlineStr">
         <is>
-          <t>(none)</t>
-        </is>
-      </c>
-      <c r="O19" s="11" t="n"/>
-      <c r="P19" s="11" t="n"/>
+          <t>about/iderma-care.png</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="P19" s="11" t="n">
+        <v>1024</v>
+      </c>
       <c r="Q19" s="8">
         <f>IF(O19="","Missing",IF(AND(O19&gt;=H19,P19&gt;=I19),"OK","Too small"))</f>
         <v/>
@@ -2286,33 +2286,33 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Store / office photo</t>
+          <t>Blog cover images</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Optional photo of the office or a map-style picture on the Contact page (needs a small code change).</t>
+          <t>A cover picture for each article (the site does not show one yet; a small code change adds it).</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>900</v>
+        <v>630</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>1200</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>675</v>
+        <v>630</v>
       </c>
       <c r="J20" s="8">
         <f>IF(OR(G20="",G20=0),"",ROUND(F20/G20,2)&amp;" : 1")</f>
@@ -2325,12 +2325,12 @@
       </c>
       <c r="L20" s="9" t="inlineStr">
         <is>
-          <t>300 KB</t>
+          <t>250 KB each</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Landscape 16:9. Helps trust for first-time buyers.</t>
+          <t>Landscape 1.91:1, one per post, no text baked in. Also used as the link preview image when the article is shared.</t>
         </is>
       </c>
       <c r="N20" s="10" t="inlineStr">
@@ -2359,33 +2359,33 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Instagram / Facebook post images</t>
+          <t>Store / office photo</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Posts for the three social accounts, to bring visitors to the site.</t>
+          <t>Optional photo of the office or a map-style picture on the Contact page (needs a small code change).</t>
         </is>
       </c>
       <c r="E21" s="8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1080</v>
+        <v>1600</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>1350</v>
+        <v>900</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>1080</v>
+        <v>1200</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>1080</v>
+        <v>675</v>
       </c>
       <c r="J21" s="8">
         <f>IF(OR(G21="",G21=0),"",ROUND(F21/G21,2)&amp;" : 1")</f>
@@ -2393,17 +2393,17 @@
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>JPG or PNG</t>
+          <t>JPG</t>
         </is>
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>1 MB each</t>
+          <t>300 KB</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>Portrait 4:5 is best for the feed. Plan about 12 for the first month. Keep the logo in one consistent corner.</t>
+          <t>Landscape 16:9. Helps trust for first-time buyers.</t>
         </is>
       </c>
       <c r="N21" s="10" t="inlineStr">
@@ -2437,28 +2437,28 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>TikTok / Reels covers</t>
+          <t>Instagram / Facebook post images</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Cover frames for videos on TikTok and Instagram Reels.</t>
+          <t>Posts for the three social accounts, to bring visitors to the site.</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>1080</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>1920</v>
+        <v>1350</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>1080</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>1920</v>
+        <v>1080</v>
       </c>
       <c r="J22" s="8">
         <f>IF(OR(G22="",G22=0),"",ROUND(F22/G22,2)&amp;" : 1")</f>
@@ -2466,17 +2466,17 @@
       </c>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>JPG</t>
+          <t>JPG or PNG</t>
         </is>
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>500 KB each</t>
+          <t>1 MB each</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>9:16. Keep text in the middle 60% - the app overlays buttons on the edges.</t>
+          <t>Portrait 4:5 is best for the feed. Plan about 12 for the first month. Keep the logo in one consistent corner.</t>
         </is>
       </c>
       <c r="N22" s="10" t="inlineStr">
@@ -2499,9 +2499,82 @@
       <c r="T22" s="12" t="n"/>
       <c r="U22" s="10" t="inlineStr"/>
     </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>TikTok / Reels covers</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Cover frames for videos on TikTok and Instagram Reels.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>1920</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>1920</v>
+      </c>
+      <c r="J23" s="8">
+        <f>IF(OR(G23="",G23=0),"",ROUND(F23/G23,2)&amp;" : 1")</f>
+        <v/>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>JPG</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>500 KB each</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>9:16. Keep text in the middle 60% - the app overlays buttons on the edges.</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="n"/>
+      <c r="P23" s="11" t="n"/>
+      <c r="Q23" s="8">
+        <f>IF(O23="","Missing",IF(AND(O23&gt;=H23,P23&gt;=I23),"OK","Too small"))</f>
+        <v/>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="S23" s="10" t="inlineStr"/>
+      <c r="T23" s="12" t="n"/>
+      <c r="U23" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U22"/>
-  <conditionalFormatting sqref="Q2:Q22">
+  <autoFilter ref="A1:U23"/>
+  <conditionalFormatting sqref="Q2:Q23">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2512,13 +2585,13 @@
       <formula>"Missing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R22">
+  <conditionalFormatting sqref="R2:R23">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>OR(R2="Live on site",R2="Approved")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="R2:R22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,In progress,Delivered,Approved,Live on site,Not needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2533,7 +2606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H19"/>
+  <dimension ref="B2:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2593,7 +2666,7 @@
     <row r="5">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Hero banner</t>
+          <t>Hero banner - desktop / tablet</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -2630,44 +2703,44 @@
     <row r="6">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Product photo</t>
+          <t>Hero banner - phone</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>1 : 1 (square)</t>
+          <t>3 : 4 (tall)</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>2000 x 2000</t>
+          <t>1080 x 1440</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>1000 x 1000</t>
+          <t>720 x 960</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>JPG / PNG</t>
+          <t>JPG / WebP</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>under 500 KB</t>
+          <t>under 300 KB</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
         <is>
-          <t>Product page gallery, product cards, cart</t>
+          <t>Home page banner on phones</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Category circle</t>
+          <t>Product photo</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -2677,12 +2750,12 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>800 x 800</t>
+          <t>2000 x 2000</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>400 x 400</t>
+          <t>1000 x 1000</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -2692,267 +2765,304 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>under 150 KB</t>
+          <t>under 500 KB</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>Home page circles</t>
+          <t>Product page gallery, product cards, cart</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Full-screen story / reel cover</t>
+          <t>Category circle</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>9 : 16 (tall)</t>
+          <t>1 : 1 (square)</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>1080 x 1920</t>
+          <t>800 x 800</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>720 x 1280</t>
+          <t>400 x 400</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>JPG / MP4</t>
+          <t>JPG / PNG</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>photo under 500 KB, video under 40 MB</t>
+          <t>under 150 KB</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
-          <t>Story viewer, TikTok and Reels</t>
+          <t>Home page circles</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Landscape video</t>
+          <t>Full-screen story / reel cover</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>16 : 9</t>
+          <t>9 : 16 (tall)</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>1920 x 1080</t>
+          <t>1080 x 1920</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>1280 x 720</t>
+          <t>720 x 1280</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
-          <t>MP4 (H.264)</t>
+          <t>JPG / MP4</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>under 40 MB</t>
+          <t>photo under 500 KB, video under 40 MB</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>Product page video player</t>
+          <t>Story viewer, TikTok and Reels</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Share / blog cover image</t>
+          <t>Landscape video</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>1.91 : 1</t>
+          <t>16 : 9</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>1200 x 630</t>
+          <t>1920 x 1080</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>1200 x 630</t>
+          <t>1280 x 720</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>JPG</t>
+          <t>MP4 (H.264)</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>under 250 KB</t>
+          <t>under 40 MB</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>Link previews on WhatsApp, Facebook; blog covers</t>
+          <t>Product page video player</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Share / blog cover image</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>wide, transparent</t>
+          <t>1.91 : 1</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>1200 x 320</t>
+          <t>1200 x 630</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>464 x 128</t>
+          <t>1200 x 630</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>PNG / SVG</t>
+          <t>JPG</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>under 300 KB</t>
+          <t>under 250 KB</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>Header on every page</t>
+          <t>Link previews on WhatsApp, Facebook; blog covers</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Favicon / square logo</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>1 : 1</t>
+          <t>wide, transparent</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>512 x 512</t>
+          <t>1200 x 320</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>256 x 256</t>
+          <t>464 x 128</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>PNG / SVG</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>under 100 KB</t>
+          <t>under 300 KB</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>Browser tab, Google, social profiles</t>
+          <t>Header on every page</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="15" t="inlineStr">
         <is>
+          <t>Favicon / square logo</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>1 : 1</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>512 x 512</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>256 x 256</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>under 100 KB</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Browser tab, Google, social profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="15" t="inlineStr">
+        <is>
           <t>Social feed post</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>4 : 5 (portrait)</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>1080 x 1350</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>1080 x 1080</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>JPG / PNG</t>
         </is>
       </c>
-      <c r="G13" s="16" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>under 1 MB</t>
         </is>
       </c>
-      <c r="H13" s="16" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>Instagram / Facebook feed</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Why "2x": phones and laptops with sharp screens show 2 pixels for every 1 on-screen pixel, so an image shown at 1200 px wide should be 2400 px wide to stay crisp.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Compress before uploading (squoosh.app or tinypng.com are free). Large images slow the site down, and speed affects Google ranking.</t>
+          <t>Why "2x": phones and laptops with sharp screens show 2 pixels for every 1 on-screen pixel, so an image shown at 1200 px wide should be 2400 px wide to stay crisp.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Name files with plain words: hero-mighty-patch-front.jpg, not IMG_4023.jpg. It helps Google Images.</t>
+          <t>Compress before uploading (squoosh.app or tinypng.com are free). Large images slow the site down, and speed affects Google ranking.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Name files with plain words: hero-mighty-patch-front.jpg, not IMG_4023.jpg. It helps Google Images.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Every picture should also have a short description (alt text) when you add it in the admin, such as "Hero Mighty Patch Invisible+ pack on a white background".</t>
         </is>
@@ -2961,7 +3071,7 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B20:H20"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B18:H18"/>
   </mergeCells>
@@ -3017,11 +3127,11 @@
         </is>
       </c>
       <c r="C5" s="19">
-        <f>COUNTIF('Content plan'!$R$2:$R$22,B5)</f>
+        <f>COUNTIF('Content plan'!$R$2:$R$23,B5)</f>
         <v/>
       </c>
       <c r="D5" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$R$2:$R$22,B5)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$R$2:$R$23,B5)</f>
         <v/>
       </c>
     </row>
@@ -3032,11 +3142,11 @@
         </is>
       </c>
       <c r="C6" s="19">
-        <f>COUNTIF('Content plan'!$R$2:$R$22,B6)</f>
+        <f>COUNTIF('Content plan'!$R$2:$R$23,B6)</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$R$2:$R$22,B6)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$R$2:$R$23,B6)</f>
         <v/>
       </c>
     </row>
@@ -3047,11 +3157,11 @@
         </is>
       </c>
       <c r="C7" s="19">
-        <f>COUNTIF('Content plan'!$R$2:$R$22,B7)</f>
+        <f>COUNTIF('Content plan'!$R$2:$R$23,B7)</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$R$2:$R$22,B7)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$R$2:$R$23,B7)</f>
         <v/>
       </c>
     </row>
@@ -3062,11 +3172,11 @@
         </is>
       </c>
       <c r="C8" s="19">
-        <f>COUNTIF('Content plan'!$R$2:$R$22,B8)</f>
+        <f>COUNTIF('Content plan'!$R$2:$R$23,B8)</f>
         <v/>
       </c>
       <c r="D8" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$R$2:$R$22,B8)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$R$2:$R$23,B8)</f>
         <v/>
       </c>
     </row>
@@ -3077,11 +3187,11 @@
         </is>
       </c>
       <c r="C9" s="19">
-        <f>COUNTIF('Content plan'!$R$2:$R$22,B9)</f>
+        <f>COUNTIF('Content plan'!$R$2:$R$23,B9)</f>
         <v/>
       </c>
       <c r="D9" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$R$2:$R$22,B9)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$R$2:$R$23,B9)</f>
         <v/>
       </c>
     </row>
@@ -3092,11 +3202,11 @@
         </is>
       </c>
       <c r="C10" s="19">
-        <f>COUNTIF('Content plan'!$R$2:$R$22,B10)</f>
+        <f>COUNTIF('Content plan'!$R$2:$R$23,B10)</f>
         <v/>
       </c>
       <c r="D10" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$R$2:$R$22,B10)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$R$2:$R$23,B10)</f>
         <v/>
       </c>
     </row>
@@ -3129,7 +3239,7 @@
         </is>
       </c>
       <c r="C14" s="19">
-        <f>COUNTIF('Content plan'!$Q$2:$Q$22,B14)</f>
+        <f>COUNTIF('Content plan'!$Q$2:$Q$23,B14)</f>
         <v/>
       </c>
     </row>
@@ -3140,7 +3250,7 @@
         </is>
       </c>
       <c r="C15" s="19">
-        <f>COUNTIF('Content plan'!$Q$2:$Q$22,B15)</f>
+        <f>COUNTIF('Content plan'!$Q$2:$Q$23,B15)</f>
         <v/>
       </c>
     </row>
@@ -3151,7 +3261,7 @@
         </is>
       </c>
       <c r="C16" s="19">
-        <f>COUNTIF('Content plan'!$Q$2:$Q$22,B16)</f>
+        <f>COUNTIF('Content plan'!$Q$2:$Q$23,B16)</f>
         <v/>
       </c>
     </row>
@@ -3174,7 +3284,7 @@
         </is>
       </c>
       <c r="C19" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B19)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B19)</f>
         <v/>
       </c>
     </row>
@@ -3185,7 +3295,7 @@
         </is>
       </c>
       <c r="C20" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B20)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B20)</f>
         <v/>
       </c>
     </row>
@@ -3196,7 +3306,7 @@
         </is>
       </c>
       <c r="C21" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B21)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B21)</f>
         <v/>
       </c>
     </row>
@@ -3207,7 +3317,7 @@
         </is>
       </c>
       <c r="C22" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B22)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B22)</f>
         <v/>
       </c>
     </row>
@@ -3218,7 +3328,7 @@
         </is>
       </c>
       <c r="C23" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B23)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B23)</f>
         <v/>
       </c>
     </row>
@@ -3229,7 +3339,7 @@
         </is>
       </c>
       <c r="C24" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B24)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B24)</f>
         <v/>
       </c>
     </row>
@@ -3240,7 +3350,7 @@
         </is>
       </c>
       <c r="C25" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B25)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B25)</f>
         <v/>
       </c>
     </row>
@@ -3251,7 +3361,7 @@
         </is>
       </c>
       <c r="C26" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B26)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B26)</f>
         <v/>
       </c>
     </row>
@@ -3262,7 +3372,7 @@
         </is>
       </c>
       <c r="C27" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B27)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B27)</f>
         <v/>
       </c>
     </row>
@@ -3273,7 +3383,7 @@
         </is>
       </c>
       <c r="C28" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B28)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B28)</f>
         <v/>
       </c>
     </row>
@@ -3284,7 +3394,7 @@
         </is>
       </c>
       <c r="C29" s="19">
-        <f>SUMIFS('Content plan'!$E$2:$E$22,'Content plan'!$B$2:$B$22,B29)</f>
+        <f>SUMIFS('Content plan'!$E$2:$E$23,'Content plan'!$B$2:$B$23,B29)</f>
         <v/>
       </c>
     </row>

</xml_diff>